<commit_message>
Save verified Fishing native articy project
</commit_message>
<xml_diff>
--- a/stories/fishing/articy/fishing-import-fixed.xlsx
+++ b/stories/fishing/articy/fishing-import-fixed.xlsx
@@ -10,7 +10,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="26">
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="30">
   <x:si>
     <x:t xml:space="preserve">Object Type:</x:t>
   </x:si>
@@ -88,6 +88,18 @@
   </x:si>
   <x:si>
     <x:t/>
+  </x:si>
+  <x:si>
+    <x:t>Fishing - Fog Sea</x:t>
+  </x:si>
+  <x:si>
+    <x:t>477a5936-34e3-4e8b-9e28-c9ba790e884c</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Fishing - Fog Sea</x:t>
+  </x:si>
+  <x:si>
+    <x:t>477a5936-34e3-4e8b-9e28-c9ba790e884c</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -524,7 +536,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="D1" s="1" t="s">
-        <x:v>3</x:v>
+        <x:v>26</x:v>
       </x:c>
     </x:row>
     <x:row r="2" s="1" customFormat="1">
@@ -538,7 +550,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>6</x:v>
+        <x:v>27</x:v>
       </x:c>
     </x:row>
     <x:row r="3" s="1" customFormat="1">
@@ -731,7 +743,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="D1" s="1" t="s">
-        <x:v>3</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="2" s="1" customFormat="1">
@@ -745,7 +757,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>6</x:v>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
     <x:row r="3" s="1" customFormat="1">

</xml_diff>